<commit_message>
named 'charts' to update raw file
</commit_message>
<xml_diff>
--- a/Chanthadara_territory_charts.xlsx
+++ b/Chanthadara_territory_charts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chimm\Documents\DATA_Labs\Capstone_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1F053916-A30C-4763-9ED9-FD97973D3973}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E5B8D8A7-2F6C-4FA6-A91D-9F5052FC9699}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{4F9622DB-3F0B-4399-96EC-3CBDB6BB25F8}"/>
   </bookViews>
@@ -422,6 +422,32 @@
           </c:extLst>
         </c:dLbl>
       </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent6">
+              <a:lumMod val="75000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
     </c:pivotFmts>
     <c:plotArea>
       <c:layout/>
@@ -476,6 +502,46 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-10B4-417C-9032-423E5AD0D6F4}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="10"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000000-10B4-417C-9032-423E5AD0D6F4}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
           <c:dLbls>
             <c:spPr>
               <a:noFill/>
@@ -1709,6 +1775,30 @@
           </c:extLst>
         </c:dLbl>
       </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent3"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
     </c:pivotFmts>
     <c:plotArea>
       <c:layout/>
@@ -1740,6 +1830,44 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000000-EA02-4C3C-A9BC-5B159CADE053}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="5"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-EA02-4C3C-A9BC-5B159CADE053}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
           <c:cat>
             <c:strRef>
               <c:f>Findings_Chart!$A$48:$A$54</c:f>
@@ -7816,6 +7944,194 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A6B0FE92-A8F0-44F2-81AE-8F660C0D359C}" name="PivotTable7" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9" rowHeaderCaption="Categories">
+  <location ref="A47:B54" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="5">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0" sortType="descending">
+      <items count="7">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="7">
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Average Transactions" fld="4" subtotal="average" baseField="2" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="3">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="2">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{CD5EED47-6634-433F-8246-8166C77A8301}" name="PivotTable6" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7" rowHeaderCaption="Territory">
+  <location ref="A7:B10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="2">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="3">
+        <item x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="% of Total_Revenue" fld="1" showDataAs="percentOfTotal" baseField="0" baseItem="0" numFmtId="10"/>
+  </dataFields>
+  <chartFormats count="3">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="2">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="3">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4F5F414B-C686-4F7F-BA97-F099CE7B7DB1}" name="PivotTable4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="18" rowHeaderCaption="Store Location">
   <location ref="A25:B37" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="3">
@@ -7924,146 +8240,6 @@
   <dataFields count="1">
     <dataField name="% of Revenue for Texas" fld="2" showDataAs="percentOfTotal" baseField="1" baseItem="4" numFmtId="10"/>
   </dataFields>
-  <chartFormats count="1">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A6B0FE92-A8F0-44F2-81AE-8F660C0D359C}" name="PivotTable7" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9" rowHeaderCaption="Categories">
-  <location ref="A47:B54" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="5">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0" sortType="descending">
-      <items count="7">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item t="default"/>
-      </items>
-      <autoSortScope>
-        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
-          <references count="1">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </autoSortScope>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="2"/>
-  </rowFields>
-  <rowItems count="7">
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Average Transactions" fld="4" subtotal="average" baseField="2" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="1">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{CD5EED47-6634-433F-8246-8166C77A8301}" name="PivotTable6" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7" rowHeaderCaption="Territory">
-  <location ref="A7:B10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="2">
-    <pivotField axis="axisRow" showAll="0">
-      <items count="3">
-        <item x="1"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField dataField="1" showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="% of Total_Revenue" fld="1" showDataAs="percentOfTotal" baseField="0" baseItem="0" numFmtId="10"/>
-  </dataFields>
   <chartFormats count="3">
     <chartFormat chart="0" format="0" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
@@ -8074,26 +8250,26 @@
         </references>
       </pivotArea>
     </chartFormat>
+    <chartFormat chart="0" format="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="6"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
     <chartFormat chart="0" format="2">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
           </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="3">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="1"/>
+          <reference field="1" count="1" selected="0">
+            <x v="4"/>
           </reference>
         </references>
       </pivotArea>

</xml_diff>